<commit_message>
Fixing ambigous translations of category bodega
</commit_message>
<xml_diff>
--- a/csv/categories_subcategories_grocery_translations.xlsx
+++ b/csv/categories_subcategories_grocery_translations.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="250">
   <si>
     <t>category_es</t>
   </si>
@@ -418,12 +418,6 @@
     <t>Baby food</t>
   </si>
   <si>
-    <t>Wine</t>
-  </si>
-  <si>
-    <t>Wine shop</t>
-  </si>
-  <si>
     <t>Cocoa, coffee and herbal teas</t>
   </si>
   <si>
@@ -463,9 +457,6 @@
     <t>Juices</t>
   </si>
   <si>
-    <t>Translated with DeepL.com (free version)</t>
-  </si>
-  <si>
     <t>Oil, vinegar and salt</t>
   </si>
   <si>
@@ -535,9 +526,6 @@
     <t>Non-alcoholic beer</t>
   </si>
   <si>
-    <t>Liqueurs</t>
-  </si>
-  <si>
     <t>Cider and cava</t>
   </si>
   <si>
@@ -770,6 +758,12 @@
   </si>
   <si>
     <t>Tomato and other flavours</t>
+  </si>
+  <si>
+    <t>Beer, wine &amp; spirits</t>
+  </si>
+  <si>
+    <t>Spirits</t>
   </si>
 </sst>
 </file>
@@ -1111,7 +1105,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D112"/>
+  <dimension ref="A1:D109"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.7109375" bestFit="1" customWidth="1"/>
@@ -1144,7 +1138,7 @@
         <v>128</v>
       </c>
       <c r="D2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1158,7 +1152,7 @@
         <v>128</v>
       </c>
       <c r="D3" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1172,7 +1166,7 @@
         <v>128</v>
       </c>
       <c r="D4" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1186,7 +1180,7 @@
         <v>128</v>
       </c>
       <c r="D5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1200,7 +1194,7 @@
         <v>129</v>
       </c>
       <c r="D6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1214,7 +1208,7 @@
         <v>129</v>
       </c>
       <c r="D7" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1228,7 +1222,7 @@
         <v>129</v>
       </c>
       <c r="D8" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1242,7 +1236,7 @@
         <v>129</v>
       </c>
       <c r="D9" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1256,7 +1250,7 @@
         <v>129</v>
       </c>
       <c r="D10" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1270,7 +1264,7 @@
         <v>129</v>
       </c>
       <c r="D11" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1284,7 +1278,7 @@
         <v>130</v>
       </c>
       <c r="D12" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1298,7 +1292,7 @@
         <v>130</v>
       </c>
       <c r="D13" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1312,7 +1306,7 @@
         <v>130</v>
       </c>
       <c r="D14" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1326,7 +1320,7 @@
         <v>131</v>
       </c>
       <c r="D15" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1340,7 +1334,7 @@
         <v>131</v>
       </c>
       <c r="D16" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1354,7 +1348,7 @@
         <v>131</v>
       </c>
       <c r="D17" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1368,7 +1362,7 @@
         <v>132</v>
       </c>
       <c r="D18" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1382,7 +1376,7 @@
         <v>132</v>
       </c>
       <c r="D19" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -1410,7 +1404,7 @@
         <v>132</v>
       </c>
       <c r="D21" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -1424,7 +1418,7 @@
         <v>132</v>
       </c>
       <c r="D22" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -1438,7 +1432,7 @@
         <v>132</v>
       </c>
       <c r="D23" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1463,10 +1457,10 @@
         <v>42</v>
       </c>
       <c r="C25" t="s">
-        <v>134</v>
+        <v>248</v>
       </c>
       <c r="D25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -1477,10 +1471,10 @@
         <v>41</v>
       </c>
       <c r="C26" t="s">
-        <v>134</v>
+        <v>248</v>
       </c>
       <c r="D26" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1491,10 +1485,10 @@
         <v>40</v>
       </c>
       <c r="C27" t="s">
-        <v>134</v>
+        <v>248</v>
       </c>
       <c r="D27" t="s">
-        <v>173</v>
+        <v>249</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1505,10 +1499,10 @@
         <v>39</v>
       </c>
       <c r="C28" t="s">
-        <v>134</v>
+        <v>248</v>
       </c>
       <c r="D28" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1519,10 +1513,10 @@
         <v>38</v>
       </c>
       <c r="C29" t="s">
-        <v>134</v>
+        <v>248</v>
       </c>
       <c r="D29" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1533,10 +1527,10 @@
         <v>37</v>
       </c>
       <c r="C30" t="s">
-        <v>134</v>
+        <v>248</v>
       </c>
       <c r="D30" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1547,10 +1541,10 @@
         <v>36</v>
       </c>
       <c r="C31" t="s">
-        <v>135</v>
+        <v>248</v>
       </c>
       <c r="D31" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1561,10 +1555,10 @@
         <v>35</v>
       </c>
       <c r="C32" t="s">
-        <v>135</v>
+        <v>248</v>
       </c>
       <c r="D32" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -1575,10 +1569,10 @@
         <v>34</v>
       </c>
       <c r="C33" t="s">
-        <v>135</v>
+        <v>248</v>
       </c>
       <c r="D33" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1589,10 +1583,10 @@
         <v>44</v>
       </c>
       <c r="C34" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D34" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -1603,10 +1597,10 @@
         <v>45</v>
       </c>
       <c r="C35" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D35" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -1617,10 +1611,10 @@
         <v>46</v>
       </c>
       <c r="C36" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D36" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1631,10 +1625,10 @@
         <v>47</v>
       </c>
       <c r="C37" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D37" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1645,10 +1639,10 @@
         <v>48</v>
       </c>
       <c r="C38" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D38" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1659,10 +1653,10 @@
         <v>58</v>
       </c>
       <c r="C39" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D39" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -1673,10 +1667,10 @@
         <v>57</v>
       </c>
       <c r="C40" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D40" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1687,10 +1681,10 @@
         <v>56</v>
       </c>
       <c r="C41" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D41" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1701,10 +1695,10 @@
         <v>55</v>
       </c>
       <c r="C42" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D42" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1715,10 +1709,10 @@
         <v>54</v>
       </c>
       <c r="C43" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D43" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -1729,10 +1723,10 @@
         <v>53</v>
       </c>
       <c r="C44" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D44" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -1743,10 +1737,10 @@
         <v>52</v>
       </c>
       <c r="C45" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D45" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -1757,10 +1751,10 @@
         <v>51</v>
       </c>
       <c r="C46" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D46" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -1771,10 +1765,10 @@
         <v>50</v>
       </c>
       <c r="C47" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D47" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -1785,10 +1779,10 @@
         <v>60</v>
       </c>
       <c r="C48" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D48" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1799,10 +1793,10 @@
         <v>61</v>
       </c>
       <c r="C49" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D49" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1813,10 +1807,10 @@
         <v>62</v>
       </c>
       <c r="C50" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D50" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -1827,10 +1821,10 @@
         <v>72</v>
       </c>
       <c r="C51" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D51" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -1841,10 +1835,10 @@
         <v>71</v>
       </c>
       <c r="C52" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D52" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -1855,10 +1849,10 @@
         <v>70</v>
       </c>
       <c r="C53" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D53" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -1869,10 +1863,10 @@
         <v>69</v>
       </c>
       <c r="C54" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D54" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -1883,10 +1877,10 @@
         <v>68</v>
       </c>
       <c r="C55" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D55" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -1897,10 +1891,10 @@
         <v>67</v>
       </c>
       <c r="C56" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D56" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -1911,10 +1905,10 @@
         <v>66</v>
       </c>
       <c r="C57" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D57" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -1925,10 +1919,10 @@
         <v>65</v>
       </c>
       <c r="C58" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D58" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -1939,10 +1933,10 @@
         <v>64</v>
       </c>
       <c r="C59" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D59" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -1953,10 +1947,10 @@
         <v>81</v>
       </c>
       <c r="C60" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D60" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -1967,10 +1961,10 @@
         <v>49</v>
       </c>
       <c r="C61" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D61" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -1981,10 +1975,10 @@
         <v>80</v>
       </c>
       <c r="C62" t="s">
+        <v>138</v>
+      </c>
+      <c r="D62" t="s">
         <v>140</v>
-      </c>
-      <c r="D62" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -1995,10 +1989,10 @@
         <v>79</v>
       </c>
       <c r="C63" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D63" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -2009,10 +2003,10 @@
         <v>78</v>
       </c>
       <c r="C64" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D64" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -2023,10 +2017,10 @@
         <v>77</v>
       </c>
       <c r="C65" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D65" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -2037,7 +2031,7 @@
         <v>76</v>
       </c>
       <c r="C66" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D66" t="s">
         <v>76</v>
@@ -2051,10 +2045,10 @@
         <v>75</v>
       </c>
       <c r="C67" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D67" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -2065,10 +2059,10 @@
         <v>74</v>
       </c>
       <c r="C68" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D68" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -2079,10 +2073,10 @@
         <v>83</v>
       </c>
       <c r="C69" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D69" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -2093,10 +2087,10 @@
         <v>84</v>
       </c>
       <c r="C70" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D70" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -2107,10 +2101,10 @@
         <v>85</v>
       </c>
       <c r="C71" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D71" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -2121,10 +2115,10 @@
         <v>86</v>
       </c>
       <c r="C72" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D72" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -2135,10 +2129,10 @@
         <v>87</v>
       </c>
       <c r="C73" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D73" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -2149,10 +2143,10 @@
         <v>88</v>
       </c>
       <c r="C74" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D74" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -2163,10 +2157,10 @@
         <v>91</v>
       </c>
       <c r="C75" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D75" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -2177,10 +2171,10 @@
         <v>90</v>
       </c>
       <c r="C76" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D76" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -2191,10 +2185,10 @@
         <v>89</v>
       </c>
       <c r="C77" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D77" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -2205,10 +2199,10 @@
         <v>93</v>
       </c>
       <c r="C78" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D78" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -2219,10 +2213,10 @@
         <v>94</v>
       </c>
       <c r="C79" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D79" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -2233,10 +2227,10 @@
         <v>95</v>
       </c>
       <c r="C80" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D80" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -2247,10 +2241,10 @@
         <v>78</v>
       </c>
       <c r="C81" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D81" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -2261,10 +2255,10 @@
         <v>99</v>
       </c>
       <c r="C82" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D82" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -2275,10 +2269,10 @@
         <v>98</v>
       </c>
       <c r="C83" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D83" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -2289,10 +2283,10 @@
         <v>97</v>
       </c>
       <c r="C84" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D84" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -2303,10 +2297,10 @@
         <v>108</v>
       </c>
       <c r="C85" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D85" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -2317,10 +2311,10 @@
         <v>107</v>
       </c>
       <c r="C86" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D86" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -2331,10 +2325,10 @@
         <v>106</v>
       </c>
       <c r="C87" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D87" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -2345,10 +2339,10 @@
         <v>105</v>
       </c>
       <c r="C88" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D88" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -2359,10 +2353,10 @@
         <v>104</v>
       </c>
       <c r="C89" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D89" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -2373,10 +2367,10 @@
         <v>103</v>
       </c>
       <c r="C90" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D90" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -2387,10 +2381,10 @@
         <v>102</v>
       </c>
       <c r="C91" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D91" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -2401,10 +2395,10 @@
         <v>101</v>
       </c>
       <c r="C92" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D92" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -2415,10 +2409,10 @@
         <v>112</v>
       </c>
       <c r="C93" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D93" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -2429,7 +2423,7 @@
         <v>76</v>
       </c>
       <c r="C94" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D94" t="s">
         <v>76</v>
@@ -2443,10 +2437,10 @@
         <v>111</v>
       </c>
       <c r="C95" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D95" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -2457,10 +2451,10 @@
         <v>110</v>
       </c>
       <c r="C96" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D96" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -2471,10 +2465,10 @@
         <v>122</v>
       </c>
       <c r="C97" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D97" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -2485,10 +2479,10 @@
         <v>121</v>
       </c>
       <c r="C98" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D98" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -2499,10 +2493,10 @@
         <v>120</v>
       </c>
       <c r="C99" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D99" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -2513,10 +2507,10 @@
         <v>119</v>
       </c>
       <c r="C100" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D100" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -2527,10 +2521,10 @@
         <v>118</v>
       </c>
       <c r="C101" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D101" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -2541,10 +2535,10 @@
         <v>117</v>
       </c>
       <c r="C102" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D102" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -2555,10 +2549,10 @@
         <v>116</v>
       </c>
       <c r="C103" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D103" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -2569,10 +2563,10 @@
         <v>115</v>
       </c>
       <c r="C104" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D104" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -2583,10 +2577,10 @@
         <v>114</v>
       </c>
       <c r="C105" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D105" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -2597,10 +2591,10 @@
         <v>126</v>
       </c>
       <c r="C106" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D106" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -2611,10 +2605,10 @@
         <v>125</v>
       </c>
       <c r="C107" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D107" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -2625,10 +2619,10 @@
         <v>124</v>
       </c>
       <c r="C108" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D108" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -2639,18 +2633,10 @@
         <v>123</v>
       </c>
       <c r="C109" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D109" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C112" t="s">
-        <v>149</v>
-      </c>
-      <c r="D112" t="s">
-        <v>149</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reviewing and fixing translations of cat & subcat
</commit_message>
<xml_diff>
--- a/csv/categories_subcategories_grocery_translations.xlsx
+++ b/csv/categories_subcategories_grocery_translations.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="251">
   <si>
     <t>category_es</t>
   </si>
@@ -400,72 +400,21 @@
     <t>Zumos</t>
   </si>
   <si>
-    <t>Oil, spices and sauces</t>
-  </si>
-  <si>
-    <t>Water and soft drinks</t>
-  </si>
-  <si>
     <t>Snacks</t>
   </si>
   <si>
-    <t>Rice, pulses and pasta</t>
-  </si>
-  <si>
-    <t>Sugar, sweets and chocolate</t>
-  </si>
-  <si>
     <t>Baby food</t>
   </si>
   <si>
-    <t>Cocoa, coffee and herbal teas</t>
-  </si>
-  <si>
     <t>Meat</t>
   </si>
   <si>
-    <t>Cereals and biscuits</t>
-  </si>
-  <si>
-    <t>Cold cuts and cheeses</t>
-  </si>
-  <si>
-    <t>Frozen foods</t>
-  </si>
-  <si>
-    <t>Tinned food, stocks and soups</t>
-  </si>
-  <si>
-    <t>Fruit and vegetables</t>
-  </si>
-  <si>
-    <t>Eggs, milk and butter</t>
-  </si>
-  <si>
-    <t>Seafood and fish</t>
-  </si>
-  <si>
-    <t>Bread and pastries</t>
-  </si>
-  <si>
-    <t>Pizzas and ready meals</t>
-  </si>
-  <si>
-    <t>Desserts and yoghurts</t>
-  </si>
-  <si>
     <t>Juices</t>
   </si>
   <si>
-    <t>Oil, vinegar and salt</t>
-  </si>
-  <si>
     <t>Spices</t>
   </si>
   <si>
-    <t>Mayonnaise, ketchup and mustard</t>
-  </si>
-  <si>
     <t>Other sauces</t>
   </si>
   <si>
@@ -475,207 +424,54 @@
     <t>Isotonic and energy drinks</t>
   </si>
   <si>
-    <t>Cola</t>
-  </si>
-  <si>
-    <t>Orange and lemon soft drinks</t>
-  </si>
-  <si>
-    <t>Tonic water and bitters</t>
-  </si>
-  <si>
-    <t>Iced tea and still tea</t>
-  </si>
-  <si>
-    <t>Olives and pickles</t>
-  </si>
-  <si>
-    <t>Nuts and dried fruit</t>
-  </si>
-  <si>
-    <t>Crisps and snacks</t>
-  </si>
-  <si>
     <t>Rice</t>
   </si>
   <si>
     <t>Pulses</t>
   </si>
   <si>
-    <t>Pasta and noodles</t>
-  </si>
-  <si>
-    <t>Sugar and sweetener</t>
-  </si>
-  <si>
-    <t>Chewing gum and sweets</t>
-  </si>
-  <si>
-    <t>Confectionery</t>
-  </si>
-  <si>
-    <t>Jam and honey</t>
-  </si>
-  <si>
-    <t>Nougat</t>
-  </si>
-  <si>
     <t>Beer</t>
   </si>
   <si>
-    <t>Non-alcoholic beer</t>
-  </si>
-  <si>
-    <t>Cider and cava</t>
-  </si>
-  <si>
-    <t>Tinto de verano and sangria</t>
-  </si>
-  <si>
     <t>White wine</t>
   </si>
   <si>
-    <t>Lambrusco and sparkling wine</t>
-  </si>
-  <si>
-    <t>Rosé wine</t>
-  </si>
-  <si>
     <t>Red wine</t>
   </si>
   <si>
-    <t>Instant cocoa and drinking chocolate</t>
-  </si>
-  <si>
-    <t>Coffee capsules and single-serve pods</t>
-  </si>
-  <si>
-    <t>Ground coffee and coffee beans</t>
-  </si>
-  <si>
-    <t>Instant coffee and other drinks</t>
-  </si>
-  <si>
-    <t>Tea and herbal teas</t>
-  </si>
-  <si>
-    <t>Ready meals</t>
-  </si>
-  <si>
-    <t>Poultry and chicken</t>
-  </si>
-  <si>
     <t>Frozen meat</t>
   </si>
   <si>
     <t>Pork</t>
   </si>
   <si>
-    <t>Rabbit and lamb</t>
-  </si>
-  <si>
     <t>Sausages</t>
   </si>
   <si>
-    <t>Burgers and minced meat products</t>
-  </si>
-  <si>
     <t>Beef</t>
   </si>
   <si>
-    <t>Breaded and processed foods</t>
-  </si>
-  <si>
     <t>Cereals</t>
   </si>
   <si>
     <t>Biscuits</t>
   </si>
   <si>
-    <t>Pancakes</t>
-  </si>
-  <si>
-    <t>Poultry and cooked ham</t>
-  </si>
-  <si>
-    <t>Bacon and sausages</t>
-  </si>
-  <si>
-    <t>Chopped meat and mortadella</t>
-  </si>
-  <si>
-    <t>Cured sausages</t>
-  </si>
-  <si>
     <t>Serrano ham</t>
   </si>
   <si>
-    <t>Pâté and sobrasada</t>
-  </si>
-  <si>
-    <t>Mature, semi-mature and soft cheese</t>
-  </si>
-  <si>
-    <t>Sliced, grated and portioned cheese</t>
-  </si>
-  <si>
-    <t>Spreadable, fresh and speciality cheeses</t>
-  </si>
-  <si>
-    <t>Rice and pasta</t>
-  </si>
-  <si>
     <t>Ice cream</t>
   </si>
   <si>
-    <t>Shellfish</t>
-  </si>
-  <si>
     <t>Fish</t>
   </si>
   <si>
-    <t>Battered foods</t>
-  </si>
-  <si>
-    <t>Cakes and churros</t>
-  </si>
-  <si>
-    <t>Tuna and other tinned fish</t>
-  </si>
-  <si>
-    <t>Cockles and mussels</t>
-  </si>
-  <si>
-    <t>Tinned fruit and vegetables</t>
-  </si>
-  <si>
-    <t>Gazpacho and cream soups</t>
-  </si>
-  <si>
-    <t>Soup and stock</t>
-  </si>
-  <si>
-    <t>Tomatoes</t>
-  </si>
-  <si>
-    <t>Fruit</t>
-  </si>
-  <si>
-    <t>Lettuce and ready-made salad</t>
-  </si>
-  <si>
     <t>Vegetables</t>
   </si>
   <si>
     <t>Eggs</t>
   </si>
   <si>
-    <t>Milk and plant-based drinks</t>
-  </si>
-  <si>
-    <t>Butter and margarine</t>
-  </si>
-  <si>
     <t>Seafood</t>
   </si>
   <si>
@@ -685,36 +481,9 @@
     <t>Fresh fish</t>
   </si>
   <si>
-    <t>Salted and smoked fish</t>
-  </si>
-  <si>
-    <t>Baked pastries</t>
-  </si>
-  <si>
     <t>Packaged pastries</t>
   </si>
   <si>
-    <t>Flour and baking mixes</t>
-  </si>
-  <si>
-    <t>Baked bread</t>
-  </si>
-  <si>
-    <t>Sliced bread and other specialities</t>
-  </si>
-  <si>
-    <t>Toasted and breadcrumbs</t>
-  </si>
-  <si>
-    <t>Breadsticks, bread rings and croutons</t>
-  </si>
-  <si>
-    <t>Cakes and pastries</t>
-  </si>
-  <si>
-    <t>Ready-to-eat</t>
-  </si>
-  <si>
     <t>Hot ready meals</t>
   </si>
   <si>
@@ -724,46 +493,280 @@
     <t>Bifidus</t>
   </si>
   <si>
-    <t>Custard and flan</t>
-  </si>
-  <si>
-    <t>Jelly and other desserts</t>
-  </si>
-  <si>
-    <t>Soya desserts</t>
-  </si>
-  <si>
-    <t>Low-fat yoghurts</t>
-  </si>
-  <si>
-    <t>Greek yoghurts</t>
-  </si>
-  <si>
-    <t>Liquid yoghurts</t>
-  </si>
-  <si>
-    <t>Natural and flavoured yoghurts</t>
-  </si>
-  <si>
-    <t>Yoghurts and desserts for children</t>
-  </si>
-  <si>
     <t>Assorted fruit</t>
   </si>
   <si>
-    <t>Peach and pineapple</t>
-  </si>
-  <si>
     <t>Orange</t>
   </si>
   <si>
-    <t>Tomato and other flavours</t>
-  </si>
-  <si>
     <t>Beer, wine &amp; spirits</t>
   </si>
   <si>
     <t>Spirits</t>
+  </si>
+  <si>
+    <t>Cola drinks</t>
+  </si>
+  <si>
+    <t>Orange &amp; lemon soft drinks</t>
+  </si>
+  <si>
+    <t>Tonic &amp; bitter</t>
+  </si>
+  <si>
+    <t>Still &amp; tea soft drinks</t>
+  </si>
+  <si>
+    <t>Olives &amp; pickles</t>
+  </si>
+  <si>
+    <t>Nuts, seeds &amp; dried fruit</t>
+  </si>
+  <si>
+    <t>Potato crisp &amp; snacks</t>
+  </si>
+  <si>
+    <t>Pasta &amp; noodles</t>
+  </si>
+  <si>
+    <t>Water &amp; soft drinks</t>
+  </si>
+  <si>
+    <t>Rice, pulses &amp; pasta</t>
+  </si>
+  <si>
+    <t>Sugar, sweets &amp; chocolate</t>
+  </si>
+  <si>
+    <t>Sugar &amp; sweetener</t>
+  </si>
+  <si>
+    <t>Chewing gum &amp; sweets</t>
+  </si>
+  <si>
+    <t>Sweets</t>
+  </si>
+  <si>
+    <t>Marmalade &amp; honey</t>
+  </si>
+  <si>
+    <t>Nougats</t>
+  </si>
+  <si>
+    <t>Baby</t>
+  </si>
+  <si>
+    <t>Alcohol-free beer</t>
+  </si>
+  <si>
+    <t>Cider &amp; cava</t>
+  </si>
+  <si>
+    <t>Tinto de verano &amp; sangria</t>
+  </si>
+  <si>
+    <t>Lambrusco &amp; sparkling wine</t>
+  </si>
+  <si>
+    <t>Rose wine</t>
+  </si>
+  <si>
+    <t>Chocolate drinks, coffee &amp; tea</t>
+  </si>
+  <si>
+    <t>Chocolate drinks &amp; hot chocolate</t>
+  </si>
+  <si>
+    <t>Coffee pods &amp; single cups</t>
+  </si>
+  <si>
+    <t>Ground coffee &amp; coffee beans</t>
+  </si>
+  <si>
+    <t>Soluble coffe &amp; other drinks</t>
+  </si>
+  <si>
+    <t>Tea &amp; infusions</t>
+  </si>
+  <si>
+    <t>Meat boxes</t>
+  </si>
+  <si>
+    <t>Poultry</t>
+  </si>
+  <si>
+    <t>Rabbit &amp; lamb</t>
+  </si>
+  <si>
+    <t>Burgers &amp; minced food</t>
+  </si>
+  <si>
+    <t>Breaded &amp; prepared meats</t>
+  </si>
+  <si>
+    <t>Cereals &amp; biscuits</t>
+  </si>
+  <si>
+    <t>Cakes</t>
+  </si>
+  <si>
+    <t>Deli &amp; cheese</t>
+  </si>
+  <si>
+    <t>Cooked poultry &amp; ham</t>
+  </si>
+  <si>
+    <t>Bacon &amp; sausages</t>
+  </si>
+  <si>
+    <t>Chopped pork &amp; mortadella</t>
+  </si>
+  <si>
+    <t>Cured meat</t>
+  </si>
+  <si>
+    <t>Pate &amp; sobrasada</t>
+  </si>
+  <si>
+    <t>Cured, semicured &amp; soft cheese</t>
+  </si>
+  <si>
+    <t>Sliced, grated &amp; portioned cheese</t>
+  </si>
+  <si>
+    <t>Spreadable cheese, fresh cheese and specialities</t>
+  </si>
+  <si>
+    <t>Frozen food</t>
+  </si>
+  <si>
+    <t>Rice &amp; pasta</t>
+  </si>
+  <si>
+    <t>Fruit &amp; vegetables</t>
+  </si>
+  <si>
+    <t>Pizza</t>
+  </si>
+  <si>
+    <t>Breaded food</t>
+  </si>
+  <si>
+    <t>Cake &amp; churros</t>
+  </si>
+  <si>
+    <t>Cans, soups &amp; creams</t>
+  </si>
+  <si>
+    <t>Tuna &amp; other fish cans</t>
+  </si>
+  <si>
+    <t>Cockles &amp; mussels</t>
+  </si>
+  <si>
+    <t>Vegetable &amp; fruit tins</t>
+  </si>
+  <si>
+    <t>Gazpacho &amp; creams</t>
+  </si>
+  <si>
+    <t>Soups &amp; stock</t>
+  </si>
+  <si>
+    <t>Tomato</t>
+  </si>
+  <si>
+    <t>Fruits</t>
+  </si>
+  <si>
+    <t>Lettuce &amp; prepared salad</t>
+  </si>
+  <si>
+    <t>Eggs, milk &amp; butter</t>
+  </si>
+  <si>
+    <t>Milk &amp; milk alternatives</t>
+  </si>
+  <si>
+    <t>Butter &amp; margarine</t>
+  </si>
+  <si>
+    <t>Seafood &amp; fish</t>
+  </si>
+  <si>
+    <t>Salted &amp; smoked fish</t>
+  </si>
+  <si>
+    <t>Bread&amp; bakery</t>
+  </si>
+  <si>
+    <t>Oven pastries</t>
+  </si>
+  <si>
+    <t>Flour &amp; baking supplies</t>
+  </si>
+  <si>
+    <t>Oven bread</t>
+  </si>
+  <si>
+    <t>Packaged sliced bread &amp; other specialities</t>
+  </si>
+  <si>
+    <t>Toasted bread &amp; breadcrumbs</t>
+  </si>
+  <si>
+    <t>Breadsticks &amp; croutons</t>
+  </si>
+  <si>
+    <t>Cakes &amp; tarts</t>
+  </si>
+  <si>
+    <t>Pizzas &amp; ready meals</t>
+  </si>
+  <si>
+    <t>Ready to eat</t>
+  </si>
+  <si>
+    <t>Desserts &amp; yoghurt</t>
+  </si>
+  <si>
+    <t>Flan &amp; custard</t>
+  </si>
+  <si>
+    <t>Jelly &amp; other desserts</t>
+  </si>
+  <si>
+    <t>Soy desserts</t>
+  </si>
+  <si>
+    <t>Low fat yoghurt</t>
+  </si>
+  <si>
+    <t>Greek yoghurt</t>
+  </si>
+  <si>
+    <t>Liquid yoghurt</t>
+  </si>
+  <si>
+    <t>Natural &amp; flavoured yoghurt</t>
+  </si>
+  <si>
+    <t>Children's yoghurt &amp; dessert</t>
+  </si>
+  <si>
+    <t>Peach &amp; pineapple</t>
+  </si>
+  <si>
+    <t>Tomato &amp; other flavours</t>
+  </si>
+  <si>
+    <t>Oil, spices &amp; sauces</t>
+  </si>
+  <si>
+    <t>Oil, vinegar &amp; salt</t>
+  </si>
+  <si>
+    <t>Mayonnaise, ketchup &amp; mustard</t>
   </si>
 </sst>
 </file>
@@ -1110,7 +1113,8 @@
   <cols>
     <col min="1" max="1" width="27.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -1135,10 +1139,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>128</v>
+        <v>248</v>
       </c>
       <c r="D2" t="s">
-        <v>147</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1149,10 +1153,10 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>128</v>
+        <v>248</v>
       </c>
       <c r="D3" t="s">
-        <v>148</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1163,10 +1167,10 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>128</v>
+        <v>248</v>
       </c>
       <c r="D4" t="s">
-        <v>149</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1177,10 +1181,10 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>128</v>
+        <v>248</v>
       </c>
       <c r="D5" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1191,10 +1195,10 @@
         <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>129</v>
+        <v>171</v>
       </c>
       <c r="D6" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1205,10 +1209,10 @@
         <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>129</v>
+        <v>171</v>
       </c>
       <c r="D7" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1219,10 +1223,10 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>129</v>
+        <v>171</v>
       </c>
       <c r="D8" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1233,10 +1237,10 @@
         <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>129</v>
+        <v>171</v>
       </c>
       <c r="D9" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1247,10 +1251,10 @@
         <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>129</v>
+        <v>171</v>
       </c>
       <c r="D10" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1261,10 +1265,10 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>129</v>
+        <v>171</v>
       </c>
       <c r="D11" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1275,10 +1279,10 @@
         <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D12" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1289,10 +1293,10 @@
         <v>18</v>
       </c>
       <c r="C13" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D13" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1303,10 +1307,10 @@
         <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D14" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1317,10 +1321,10 @@
         <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>131</v>
+        <v>172</v>
       </c>
       <c r="D15" t="s">
-        <v>160</v>
+        <v>136</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1331,10 +1335,10 @@
         <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>131</v>
+        <v>172</v>
       </c>
       <c r="D16" t="s">
-        <v>161</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1345,10 +1349,10 @@
         <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>131</v>
+        <v>172</v>
       </c>
       <c r="D17" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1359,10 +1363,10 @@
         <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>132</v>
+        <v>173</v>
       </c>
       <c r="D18" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1373,10 +1377,10 @@
         <v>29</v>
       </c>
       <c r="C19" t="s">
-        <v>132</v>
+        <v>173</v>
       </c>
       <c r="D19" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -1387,7 +1391,7 @@
         <v>28</v>
       </c>
       <c r="C20" t="s">
-        <v>132</v>
+        <v>173</v>
       </c>
       <c r="D20" t="s">
         <v>28</v>
@@ -1401,10 +1405,10 @@
         <v>27</v>
       </c>
       <c r="C21" t="s">
-        <v>132</v>
+        <v>173</v>
       </c>
       <c r="D21" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -1415,10 +1419,10 @@
         <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>132</v>
+        <v>173</v>
       </c>
       <c r="D22" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -1429,10 +1433,10 @@
         <v>25</v>
       </c>
       <c r="C23" t="s">
-        <v>132</v>
+        <v>173</v>
       </c>
       <c r="D23" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1443,10 +1447,10 @@
         <v>32</v>
       </c>
       <c r="C24" t="s">
-        <v>133</v>
+        <v>179</v>
       </c>
       <c r="D24" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1457,10 +1461,10 @@
         <v>42</v>
       </c>
       <c r="C25" t="s">
-        <v>248</v>
+        <v>161</v>
       </c>
       <c r="D25" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -1471,10 +1475,10 @@
         <v>41</v>
       </c>
       <c r="C26" t="s">
-        <v>248</v>
+        <v>161</v>
       </c>
       <c r="D26" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1485,10 +1489,10 @@
         <v>40</v>
       </c>
       <c r="C27" t="s">
-        <v>248</v>
+        <v>161</v>
       </c>
       <c r="D27" t="s">
-        <v>249</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1499,10 +1503,10 @@
         <v>39</v>
       </c>
       <c r="C28" t="s">
-        <v>248</v>
+        <v>161</v>
       </c>
       <c r="D28" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1513,10 +1517,10 @@
         <v>38</v>
       </c>
       <c r="C29" t="s">
-        <v>248</v>
+        <v>161</v>
       </c>
       <c r="D29" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1527,10 +1531,10 @@
         <v>37</v>
       </c>
       <c r="C30" t="s">
-        <v>248</v>
+        <v>161</v>
       </c>
       <c r="D30" t="s">
-        <v>172</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1541,10 +1545,10 @@
         <v>36</v>
       </c>
       <c r="C31" t="s">
-        <v>248</v>
+        <v>161</v>
       </c>
       <c r="D31" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1555,10 +1559,10 @@
         <v>35</v>
       </c>
       <c r="C32" t="s">
-        <v>248</v>
+        <v>161</v>
       </c>
       <c r="D32" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -1569,10 +1573,10 @@
         <v>34</v>
       </c>
       <c r="C33" t="s">
-        <v>248</v>
+        <v>161</v>
       </c>
       <c r="D33" t="s">
-        <v>175</v>
+        <v>140</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1583,10 +1587,10 @@
         <v>44</v>
       </c>
       <c r="C34" t="s">
-        <v>134</v>
+        <v>185</v>
       </c>
       <c r="D34" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -1597,10 +1601,10 @@
         <v>45</v>
       </c>
       <c r="C35" t="s">
-        <v>134</v>
+        <v>185</v>
       </c>
       <c r="D35" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -1611,10 +1615,10 @@
         <v>46</v>
       </c>
       <c r="C36" t="s">
-        <v>134</v>
+        <v>185</v>
       </c>
       <c r="D36" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1625,10 +1629,10 @@
         <v>47</v>
       </c>
       <c r="C37" t="s">
-        <v>134</v>
+        <v>185</v>
       </c>
       <c r="D37" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1639,10 +1643,10 @@
         <v>48</v>
       </c>
       <c r="C38" t="s">
-        <v>134</v>
+        <v>185</v>
       </c>
       <c r="D38" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1653,10 +1657,10 @@
         <v>58</v>
       </c>
       <c r="C39" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D39" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -1667,10 +1671,10 @@
         <v>57</v>
       </c>
       <c r="C40" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D40" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1681,10 +1685,10 @@
         <v>56</v>
       </c>
       <c r="C41" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D41" t="s">
-        <v>183</v>
+        <v>141</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1695,10 +1699,10 @@
         <v>55</v>
       </c>
       <c r="C42" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D42" t="s">
-        <v>184</v>
+        <v>142</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1709,10 +1713,10 @@
         <v>54</v>
       </c>
       <c r="C43" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D43" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -1723,10 +1727,10 @@
         <v>53</v>
       </c>
       <c r="C44" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D44" t="s">
-        <v>186</v>
+        <v>143</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -1737,10 +1741,10 @@
         <v>52</v>
       </c>
       <c r="C45" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D45" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -1751,10 +1755,10 @@
         <v>51</v>
       </c>
       <c r="C46" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D46" t="s">
-        <v>188</v>
+        <v>144</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -1765,10 +1769,10 @@
         <v>50</v>
       </c>
       <c r="C47" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D47" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -1779,10 +1783,10 @@
         <v>60</v>
       </c>
       <c r="C48" t="s">
-        <v>136</v>
+        <v>196</v>
       </c>
       <c r="D48" t="s">
-        <v>190</v>
+        <v>145</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1793,10 +1797,10 @@
         <v>61</v>
       </c>
       <c r="C49" t="s">
-        <v>136</v>
+        <v>196</v>
       </c>
       <c r="D49" t="s">
-        <v>191</v>
+        <v>146</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1807,10 +1811,10 @@
         <v>62</v>
       </c>
       <c r="C50" t="s">
-        <v>136</v>
+        <v>196</v>
       </c>
       <c r="D50" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -1821,10 +1825,10 @@
         <v>72</v>
       </c>
       <c r="C51" t="s">
-        <v>137</v>
+        <v>198</v>
       </c>
       <c r="D51" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -1835,10 +1839,10 @@
         <v>71</v>
       </c>
       <c r="C52" t="s">
-        <v>137</v>
+        <v>198</v>
       </c>
       <c r="D52" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -1849,10 +1853,10 @@
         <v>70</v>
       </c>
       <c r="C53" t="s">
-        <v>137</v>
+        <v>198</v>
       </c>
       <c r="D53" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -1863,10 +1867,10 @@
         <v>69</v>
       </c>
       <c r="C54" t="s">
-        <v>137</v>
+        <v>198</v>
       </c>
       <c r="D54" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -1877,10 +1881,10 @@
         <v>68</v>
       </c>
       <c r="C55" t="s">
-        <v>137</v>
+        <v>198</v>
       </c>
       <c r="D55" t="s">
-        <v>197</v>
+        <v>147</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -1891,10 +1895,10 @@
         <v>67</v>
       </c>
       <c r="C56" t="s">
-        <v>137</v>
+        <v>198</v>
       </c>
       <c r="D56" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -1905,10 +1909,10 @@
         <v>66</v>
       </c>
       <c r="C57" t="s">
-        <v>137</v>
+        <v>198</v>
       </c>
       <c r="D57" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -1919,10 +1923,10 @@
         <v>65</v>
       </c>
       <c r="C58" t="s">
-        <v>137</v>
+        <v>198</v>
       </c>
       <c r="D58" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -1933,10 +1937,10 @@
         <v>64</v>
       </c>
       <c r="C59" t="s">
-        <v>137</v>
+        <v>198</v>
       </c>
       <c r="D59" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -1947,10 +1951,10 @@
         <v>81</v>
       </c>
       <c r="C60" t="s">
-        <v>138</v>
+        <v>207</v>
       </c>
       <c r="D60" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -1961,10 +1965,10 @@
         <v>49</v>
       </c>
       <c r="C61" t="s">
-        <v>138</v>
+        <v>207</v>
       </c>
       <c r="D61" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -1975,10 +1979,10 @@
         <v>80</v>
       </c>
       <c r="C62" t="s">
-        <v>138</v>
+        <v>207</v>
       </c>
       <c r="D62" t="s">
-        <v>140</v>
+        <v>209</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -1989,10 +1993,10 @@
         <v>79</v>
       </c>
       <c r="C63" t="s">
-        <v>138</v>
+        <v>207</v>
       </c>
       <c r="D63" t="s">
-        <v>203</v>
+        <v>148</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -2003,10 +2007,10 @@
         <v>78</v>
       </c>
       <c r="C64" t="s">
-        <v>138</v>
+        <v>207</v>
       </c>
       <c r="D64" t="s">
-        <v>204</v>
+        <v>152</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -2017,10 +2021,10 @@
         <v>77</v>
       </c>
       <c r="C65" t="s">
-        <v>138</v>
+        <v>207</v>
       </c>
       <c r="D65" t="s">
-        <v>205</v>
+        <v>149</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -2031,10 +2035,10 @@
         <v>76</v>
       </c>
       <c r="C66" t="s">
-        <v>138</v>
+        <v>207</v>
       </c>
       <c r="D66" t="s">
-        <v>76</v>
+        <v>210</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -2045,10 +2049,10 @@
         <v>75</v>
       </c>
       <c r="C67" t="s">
-        <v>138</v>
+        <v>207</v>
       </c>
       <c r="D67" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -2059,10 +2063,10 @@
         <v>74</v>
       </c>
       <c r="C68" t="s">
-        <v>138</v>
+        <v>207</v>
       </c>
       <c r="D68" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -2073,10 +2077,10 @@
         <v>83</v>
       </c>
       <c r="C69" t="s">
-        <v>139</v>
+        <v>213</v>
       </c>
       <c r="D69" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -2087,10 +2091,10 @@
         <v>84</v>
       </c>
       <c r="C70" t="s">
-        <v>139</v>
+        <v>213</v>
       </c>
       <c r="D70" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -2101,10 +2105,10 @@
         <v>85</v>
       </c>
       <c r="C71" t="s">
-        <v>139</v>
+        <v>213</v>
       </c>
       <c r="D71" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -2115,10 +2119,10 @@
         <v>86</v>
       </c>
       <c r="C72" t="s">
-        <v>139</v>
+        <v>213</v>
       </c>
       <c r="D72" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -2129,10 +2133,10 @@
         <v>87</v>
       </c>
       <c r="C73" t="s">
-        <v>139</v>
+        <v>213</v>
       </c>
       <c r="D73" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -2143,10 +2147,10 @@
         <v>88</v>
       </c>
       <c r="C74" t="s">
-        <v>139</v>
+        <v>213</v>
       </c>
       <c r="D74" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -2157,10 +2161,10 @@
         <v>91</v>
       </c>
       <c r="C75" t="s">
-        <v>140</v>
+        <v>209</v>
       </c>
       <c r="D75" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -2171,10 +2175,10 @@
         <v>90</v>
       </c>
       <c r="C76" t="s">
-        <v>140</v>
+        <v>209</v>
       </c>
       <c r="D76" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -2185,10 +2189,10 @@
         <v>89</v>
       </c>
       <c r="C77" t="s">
-        <v>140</v>
+        <v>209</v>
       </c>
       <c r="D77" t="s">
-        <v>216</v>
+        <v>150</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -2199,10 +2203,10 @@
         <v>93</v>
       </c>
       <c r="C78" t="s">
-        <v>141</v>
+        <v>222</v>
       </c>
       <c r="D78" t="s">
-        <v>217</v>
+        <v>151</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -2213,10 +2217,10 @@
         <v>94</v>
       </c>
       <c r="C79" t="s">
-        <v>141</v>
+        <v>222</v>
       </c>
       <c r="D79" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -2227,10 +2231,10 @@
         <v>95</v>
       </c>
       <c r="C80" t="s">
-        <v>141</v>
+        <v>222</v>
       </c>
       <c r="D80" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -2241,10 +2245,10 @@
         <v>78</v>
       </c>
       <c r="C81" t="s">
-        <v>142</v>
+        <v>225</v>
       </c>
       <c r="D81" t="s">
-        <v>220</v>
+        <v>152</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -2255,10 +2259,10 @@
         <v>99</v>
       </c>
       <c r="C82" t="s">
-        <v>142</v>
+        <v>225</v>
       </c>
       <c r="D82" t="s">
-        <v>221</v>
+        <v>153</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -2269,10 +2273,10 @@
         <v>98</v>
       </c>
       <c r="C83" t="s">
-        <v>142</v>
+        <v>225</v>
       </c>
       <c r="D83" t="s">
-        <v>222</v>
+        <v>154</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -2283,10 +2287,10 @@
         <v>97</v>
       </c>
       <c r="C84" t="s">
-        <v>142</v>
+        <v>225</v>
       </c>
       <c r="D84" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -2297,10 +2301,10 @@
         <v>108</v>
       </c>
       <c r="C85" t="s">
-        <v>143</v>
+        <v>227</v>
       </c>
       <c r="D85" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -2311,10 +2315,10 @@
         <v>107</v>
       </c>
       <c r="C86" t="s">
-        <v>143</v>
+        <v>227</v>
       </c>
       <c r="D86" t="s">
-        <v>225</v>
+        <v>155</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -2325,10 +2329,10 @@
         <v>106</v>
       </c>
       <c r="C87" t="s">
-        <v>143</v>
+        <v>227</v>
       </c>
       <c r="D87" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -2339,10 +2343,10 @@
         <v>105</v>
       </c>
       <c r="C88" t="s">
-        <v>143</v>
+        <v>227</v>
       </c>
       <c r="D88" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -2353,10 +2357,10 @@
         <v>104</v>
       </c>
       <c r="C89" t="s">
-        <v>143</v>
+        <v>227</v>
       </c>
       <c r="D89" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -2367,10 +2371,10 @@
         <v>103</v>
       </c>
       <c r="C90" t="s">
-        <v>143</v>
+        <v>227</v>
       </c>
       <c r="D90" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -2381,10 +2385,10 @@
         <v>102</v>
       </c>
       <c r="C91" t="s">
-        <v>143</v>
+        <v>227</v>
       </c>
       <c r="D91" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -2395,10 +2399,10 @@
         <v>101</v>
       </c>
       <c r="C92" t="s">
-        <v>143</v>
+        <v>227</v>
       </c>
       <c r="D92" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -2409,10 +2413,10 @@
         <v>112</v>
       </c>
       <c r="C93" t="s">
-        <v>144</v>
+        <v>235</v>
       </c>
       <c r="D93" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -2423,10 +2427,10 @@
         <v>76</v>
       </c>
       <c r="C94" t="s">
-        <v>144</v>
+        <v>235</v>
       </c>
       <c r="D94" t="s">
-        <v>76</v>
+        <v>210</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -2437,10 +2441,10 @@
         <v>111</v>
       </c>
       <c r="C95" t="s">
-        <v>144</v>
+        <v>235</v>
       </c>
       <c r="D95" t="s">
-        <v>233</v>
+        <v>156</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -2451,10 +2455,10 @@
         <v>110</v>
       </c>
       <c r="C96" t="s">
-        <v>144</v>
+        <v>235</v>
       </c>
       <c r="D96" t="s">
-        <v>234</v>
+        <v>157</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -2465,10 +2469,10 @@
         <v>122</v>
       </c>
       <c r="C97" t="s">
-        <v>145</v>
+        <v>237</v>
       </c>
       <c r="D97" t="s">
-        <v>235</v>
+        <v>158</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -2479,10 +2483,10 @@
         <v>121</v>
       </c>
       <c r="C98" t="s">
-        <v>145</v>
+        <v>237</v>
       </c>
       <c r="D98" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -2493,10 +2497,10 @@
         <v>120</v>
       </c>
       <c r="C99" t="s">
-        <v>145</v>
+        <v>237</v>
       </c>
       <c r="D99" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -2507,10 +2511,10 @@
         <v>119</v>
       </c>
       <c r="C100" t="s">
-        <v>145</v>
+        <v>237</v>
       </c>
       <c r="D100" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -2521,10 +2525,10 @@
         <v>118</v>
       </c>
       <c r="C101" t="s">
-        <v>145</v>
+        <v>237</v>
       </c>
       <c r="D101" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -2535,10 +2539,10 @@
         <v>117</v>
       </c>
       <c r="C102" t="s">
-        <v>145</v>
+        <v>237</v>
       </c>
       <c r="D102" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -2549,10 +2553,10 @@
         <v>116</v>
       </c>
       <c r="C103" t="s">
-        <v>145</v>
+        <v>237</v>
       </c>
       <c r="D103" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -2563,10 +2567,10 @@
         <v>115</v>
       </c>
       <c r="C104" t="s">
-        <v>145</v>
+        <v>237</v>
       </c>
       <c r="D104" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -2577,10 +2581,10 @@
         <v>114</v>
       </c>
       <c r="C105" t="s">
-        <v>145</v>
+        <v>237</v>
       </c>
       <c r="D105" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -2591,10 +2595,10 @@
         <v>126</v>
       </c>
       <c r="C106" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="D106" t="s">
-        <v>244</v>
+        <v>159</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -2605,10 +2609,10 @@
         <v>125</v>
       </c>
       <c r="C107" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="D107" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -2619,10 +2623,10 @@
         <v>124</v>
       </c>
       <c r="C108" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="D108" t="s">
-        <v>246</v>
+        <v>160</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -2633,7 +2637,7 @@
         <v>123</v>
       </c>
       <c r="C109" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="D109" t="s">
         <v>247</v>

</xml_diff>